<commit_message>
streamline extraction logging and improve error handling
- Updated log files to reflect successful processing of 263 files across multiple processes with zero failures.
- Enhanced logging to skip already processed files, improving efficiency and reducing redundancy.
- Improved error handling for API call failures, ensuring better management of rate limits and retries.
- Cleaned up outdated debug information in logs to focus on relevant extraction details.
- Adjusted paths in scripts for consistency with the new directory structure.
</commit_message>
<xml_diff>
--- a/outputs/analysis/analysis_output/tables/part2/benefit_column_mapping.xlsx
+++ b/outputs/analysis/analysis_output/tables/part2/benefit_column_mapping.xlsx
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>426</v>
+        <v>469</v>
       </c>
       <c r="D2" t="inlineStr"/>
     </row>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1396</v>
+        <v>1224</v>
       </c>
       <c r="D3" t="inlineStr"/>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1421</v>
+        <v>1111</v>
       </c>
       <c r="D4" t="inlineStr"/>
     </row>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1220</v>
+        <v>992</v>
       </c>
       <c r="D5" t="inlineStr"/>
     </row>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1552</v>
+        <v>1476</v>
       </c>
       <c r="D6" t="inlineStr"/>
     </row>
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1525</v>
+        <v>1476</v>
       </c>
       <c r="D7" t="inlineStr"/>
     </row>
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1530</v>
+        <v>1470</v>
       </c>
       <c r="D8" t="inlineStr"/>
     </row>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1477</v>
+        <v>1284</v>
       </c>
       <c r="D9" t="inlineStr"/>
     </row>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1009</v>
+        <v>509</v>
       </c>
       <c r="D10" t="inlineStr"/>
     </row>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>969</v>
+        <v>741</v>
       </c>
       <c r="D11" t="inlineStr"/>
     </row>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1233</v>
+        <v>816</v>
       </c>
       <c r="D12" t="inlineStr"/>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1565</v>
+        <v>1458</v>
       </c>
       <c r="D13" t="inlineStr"/>
     </row>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1551</v>
+        <v>1382</v>
       </c>
       <c r="D14" t="inlineStr"/>
     </row>
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>680</v>
+        <v>836</v>
       </c>
       <c r="D15" t="inlineStr"/>
     </row>
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1529</v>
+        <v>1463</v>
       </c>
       <c r="D16" t="inlineStr"/>
     </row>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1214</v>
+        <v>933</v>
       </c>
       <c r="D17" t="inlineStr"/>
     </row>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1474</v>
+        <v>698</v>
       </c>
       <c r="D18" t="inlineStr"/>
     </row>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>826</v>
+        <v>415</v>
       </c>
       <c r="D19" t="inlineStr"/>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1327</v>
+        <v>1113</v>
       </c>
       <c r="D20" t="inlineStr"/>
     </row>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1350</v>
+        <v>1156</v>
       </c>
       <c r="D21" t="inlineStr"/>
     </row>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1541</v>
+        <v>1451</v>
       </c>
       <c r="D22" t="inlineStr"/>
     </row>
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1477</v>
+        <v>1374</v>
       </c>
       <c r="D23" t="inlineStr"/>
     </row>
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1424</v>
+        <v>1308</v>
       </c>
       <c r="D24" t="inlineStr"/>
     </row>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1425</v>
+        <v>1306</v>
       </c>
       <c r="D25" t="inlineStr"/>
     </row>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1575</v>
+        <v>1467</v>
       </c>
       <c r="D26" t="inlineStr"/>
     </row>

</xml_diff>